<commit_message>
add weighted cox models
</commit_message>
<xml_diff>
--- a/03_Output/Models/Tables/Tab_Exposure_PO_IQR.xlsx
+++ b/03_Output/Models/Tables/Tab_Exposure_PO_IQR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/jdconejeros_uc_cl/Documents/Research/Pollution_PerinatalOutcomes_Temuco26/03_Output/Models/Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_59302B3AAE327A8B70A5571423FBFADCAB4AC4BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D088DC2C-122F-AE4F-99E0-E8F4C8FA3FAF}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_59302B3AAE327A8B70A5571423FBFADCAB4AC4BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A14E4033-690E-264E-A494-B8A2FD7D7D18}"/>
   <bookViews>
-    <workbookView xWindow="-3840" yWindow="-21600" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1360" yWindow="-28800" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OR" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HR!$A$1:$N$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OR!$A$1:$N$36</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
@@ -2968,13 +2969,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" hidden="1" customWidth="1"/>
+    <col min="4" max="8" width="16.6640625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
     <col min="10" max="14" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -3023,7 +3025,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -3243,7 +3245,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>80</v>
       </c>
@@ -3463,7 +3465,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>141</v>
       </c>
@@ -3683,7 +3685,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>202</v>
       </c>
@@ -3903,7 +3905,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>263</v>
       </c>
@@ -3947,7 +3949,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>263</v>
       </c>
@@ -3991,7 +3993,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>263</v>
       </c>
@@ -4035,7 +4037,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>263</v>
       </c>
@@ -4079,7 +4081,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>263</v>
       </c>
@@ -4123,7 +4125,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>324</v>
       </c>
@@ -4167,7 +4169,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>324</v>
       </c>
@@ -4211,7 +4213,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>324</v>
       </c>
@@ -4255,7 +4257,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>324</v>
       </c>
@@ -4299,7 +4301,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>324</v>
       </c>
@@ -4343,7 +4345,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>385</v>
       </c>
@@ -4387,7 +4389,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>385</v>
       </c>
@@ -4431,7 +4433,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>385</v>
       </c>
@@ -4475,7 +4477,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>385</v>
       </c>
@@ -4519,7 +4521,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>385</v>
       </c>
@@ -4564,6 +4566,24 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N36" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Late preterm birth"/>
+        <filter val="Moderately preterm birth"/>
+        <filter val="Preterm birth"/>
+        <filter val="Very preterm birth"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Overall"/>
+        <filter val="T1"/>
+        <filter val="T2"/>
+        <filter val="T3"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4576,8 +4596,8 @@
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" hidden="1" customWidth="1"/>
+    <col min="4" max="8" width="16.6640625" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
     <col min="10" max="14" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -4626,7 +4646,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -4890,7 +4910,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>80</v>
       </c>
@@ -4934,7 +4954,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="9" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>80</v>
       </c>
@@ -4978,7 +4998,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>80</v>
       </c>
@@ -5022,7 +5042,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="11" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>80</v>
       </c>
@@ -5110,7 +5130,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="13" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>141</v>
       </c>
@@ -5154,7 +5174,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="14" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -5198,7 +5218,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="15" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -5242,7 +5262,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="16" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -5330,7 +5350,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="18" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>202</v>
       </c>
@@ -5374,7 +5394,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="19" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>202</v>
       </c>
@@ -5418,7 +5438,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="20" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>202</v>
       </c>
@@ -5462,7 +5482,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="21" spans="1:14" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>202</v>
       </c>
@@ -6170,7 +6190,18 @@
   <autoFilter ref="A1:N36" xr:uid="{00000000-0001-0000-0100-000000000000}">
     <filterColumn colId="0">
       <filters>
+        <filter val="Late preterm birth"/>
+        <filter val="Moderately preterm birth"/>
         <filter val="Preterm birth"/>
+        <filter val="Very preterm birth"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Overall"/>
+        <filter val="T1"/>
+        <filter val="T2"/>
+        <filter val="T3"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>